<commit_message>
Add cards-related block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (18):
- AGENTS.xml
- CLAUDE.xml
- CODE_OF_CONDUCT.xml
- CONTRIBUTING.xml
- README.xml
- blocks/cards-related/_cards-related.json
- component-definition.json
- component-filters.json
- component-models.json
- tools/importer/import-content-page.bundle.js
- tools/importer/import-content-page.js
- tools/importer/import-programme-landing.bundle.js
- tools/importer/import-programme-landing.js
- tools/importer/reports/get-involved/apply-for-permits/how-we-regulate.report.json
- tools/importer/reports/import-content-page.report.xlsx
- tools/importer/reports/import-programme-landing.report.xlsx
- tools/importer/reports/our-work/save-our-iconic-kiwi.report.json
- tools/importer/reports/our-work/takahe-recovery-programme.report.json
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-content-page.report.xlsx
+++ b/tools/importer/reports/import-content-page.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
   <si>
     <t>_reportFile</t>
   </si>
@@ -52,7 +52,7 @@
     <t>content-page</t>
   </si>
   <si>
-    <t>2026-07-24T02:02:32.505Z</t>
+    <t>2026-07-24T02:29:13.986Z</t>
   </si>
   <si>
     <t>Save Our Iconic Kiwi: Our work</t>
@@ -61,16 +61,34 @@
     <t>https://www.doc.govt.nz/our-work/save-our-iconic-kiwi/</t>
   </si>
   <si>
+    <t>our-work/takahe-recovery-programme.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","cards-related"]</t>
+  </si>
+  <si>
+    <t>our-work/takahe-recovery-programme</t>
+  </si>
+  <si>
+    <t>programme-landing</t>
+  </si>
+  <si>
+    <t>2026-07-24T02:26:58.454Z</t>
+  </si>
+  <si>
+    <t>Takahē Recovery Programme</t>
+  </si>
+  <si>
+    <t>https://www.doc.govt.nz/our-work/takahe-recovery-programme/</t>
+  </si>
+  <si>
     <t>get-involved/apply-for-permits/how-we-regulate.report.json</t>
   </si>
   <si>
-    <t>["hero-banner","cards-related"]</t>
-  </si>
-  <si>
     <t>get-involved/apply-for-permits/how-we-regulate</t>
   </si>
   <si>
-    <t>2026-07-24T02:02:25.301Z</t>
+    <t>2026-07-24T02:29:06.173Z</t>
   </si>
   <si>
     <t>How we regulate: Permissions</t>
@@ -465,13 +483,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
     <col min="2" max="2" width="47" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="5" max="5" width="19" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="7" width="32" customWidth="1"/>
     <col min="8" max="8" width="50" customWidth="1"/>
@@ -543,16 +561,42 @@
         <v>11</v>
       </c>
       <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
         <v>12</v>
       </c>
-      <c r="F3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H3" t="s">
-        <v>21</v>
+      <c r="F4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Import native-plants page and related-card placeholder pages
Add the doc.govt.nz "Native plants" page to the content-page template
(URL, page properties, re-bundled import script) and generate it via the
existing importer.

Add a minimal stub import script (import-stub.js) that emits a
hero-banner title-only placeholder, and use it to create the three
"Related" link targets referenced by the Native plants page:
- Attract birds to your garden
- Motukārara Wholesale Conservation Nursery
- New Zealand Threat Classification System

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-content-page.report.xlsx
+++ b/tools/importer/reports/import-content-page.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="40">
   <si>
     <t>_reportFile</t>
   </si>
@@ -37,6 +37,30 @@
     <t>url</t>
   </si>
   <si>
+    <t>nature/native-plants.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","cards-related"]</t>
+  </si>
+  <si>
+    <t>nature/native-plants</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>content-page</t>
+  </si>
+  <si>
+    <t>2026-08-07T11:35:42.758Z</t>
+  </si>
+  <si>
+    <t>New Zealand native plants: Conservation</t>
+  </si>
+  <si>
+    <t>https://www.doc.govt.nz/nature/native-plants/</t>
+  </si>
+  <si>
     <t>our-work/save-our-iconic-kiwi.report.json</t>
   </si>
   <si>
@@ -46,12 +70,6 @@
     <t>our-work/save-our-iconic-kiwi</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
-    <t>content-page</t>
-  </si>
-  <si>
     <t>2026-07-24T02:29:13.986Z</t>
   </si>
   <si>
@@ -64,16 +82,13 @@
     <t>our-work/takahe-recovery-programme.report.json</t>
   </si>
   <si>
-    <t>["hero-banner","cards-related"]</t>
-  </si>
-  <si>
     <t>our-work/takahe-recovery-programme</t>
   </si>
   <si>
     <t>programme-landing</t>
   </si>
   <si>
-    <t>2026-07-24T02:26:58.454Z</t>
+    <t>2026-07-24T02:29:21.151Z</t>
   </si>
   <si>
     <t>Takahē Recovery Programme</t>
@@ -95,6 +110,27 @@
   </si>
   <si>
     <t>https://www.doc.govt.nz/get-involved/apply-for-permits/how-we-regulate/</t>
+  </si>
+  <si>
+    <t>parks-and-recreation/places-to-go/central-north-island/places/tongariro-national-park/things-to-do/tracks/tongariro-alpine-crossing-bookings/booking-form.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","form-booking","cards-related"]</t>
+  </si>
+  <si>
+    <t>parks-and-recreation/places-to-go/central-north-island/places/tongariro-national-park/things-to-do/tracks/tongariro-alpine-crossing-bookings/booking-form</t>
+  </si>
+  <si>
+    <t>booking-form</t>
+  </si>
+  <si>
+    <t>2026-08-06T00:29:18.688Z</t>
+  </si>
+  <si>
+    <t>Tongariro Alpine Crossing booking form</t>
+  </si>
+  <si>
+    <t>https://www.doc.govt.nz/parks-and-recreation/places-to-go/central-north-island/places/tongariro-national-park/things-to-do/tracks/tongariro-alpine-crossing-bookings/booking-form/</t>
   </si>
 </sst>
 </file>
@@ -483,15 +519,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
-    <col min="2" max="2" width="47" customWidth="1"/>
-    <col min="3" max="3" width="48" customWidth="1"/>
+    <col min="2" max="2" width="48" customWidth="1"/>
+    <col min="3" max="3" width="50" customWidth="1"/>
     <col min="5" max="5" width="19" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="32" customWidth="1"/>
+    <col min="7" max="7" width="41" customWidth="1"/>
     <col min="8" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
@@ -561,33 +597,33 @@
         <v>11</v>
       </c>
       <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
         <v>19</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>20</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>21</v>
-      </c>
-      <c r="H3" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
         <v>23</v>
-      </c>
-      <c r="B4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" t="s">
-        <v>24</v>
       </c>
       <c r="D4" t="s">
         <v>11</v>
       </c>
       <c r="E4" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F4" t="s">
         <v>25</v>
@@ -597,6 +633,58 @@
       </c>
       <c r="H4" t="s">
         <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" t="s">
+        <v>31</v>
+      </c>
+      <c r="H5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>36</v>
+      </c>
+      <c r="F6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G6" t="s">
+        <v>38</v>
+      </c>
+      <c r="H6" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>